<commit_message>
Add contact, socials, location and QR shortcuts; easier navigation
- Shop phone, WhatsApp, Instagram, Facebook and Google Maps link built in
  as defaults (overridable from the sheet's الإعدادات tab; empty cells keep them)
- One-tap actions in the hero: location, call, Instagram, Facebook
- New 'زورونا' section with directions, call, socials, WhatsApp and a QR link
- Top bar: tap the logo to jump to top, pin button jumps to location
- Shorter hero so the menu shows sooner; QR page links back to the menu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FLL4Gm3gtujziqRnxdMGHJ
</commit_message>
<xml_diff>
--- a/docs/menu-template.xlsx
+++ b/docs/menu-template.xlsx
@@ -4257,12 +4257,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>96170123456</t>
+          <t>96171819311</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>رقم واتساب المقهى مع رمز البلد، أرقام فقط</t>
+          <t>رقم واتساب الذي تصله الطلبات، مع رمز البلد، أرقام فقط</t>
         </is>
       </c>
     </row>
@@ -4325,60 +4325,100 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>انستغرام</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr"/>
+          <t>الهاتف</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>71 819 311</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>اسم الحساب بدون @</t>
+          <t>رقم الاتصال الظاهر في الموقع</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>إعلان</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr"/>
+          <t>رابط الموقع</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/NZzVyibw7Cs3BuqcA</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>شريط إعلان أعلى الصفحة (اتركه فارغاً لإخفائه)</t>
+          <t>رابط Google Maps للمقهى</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>انستغرام</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/barista_alasmar</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>رابط الحساب أو اسمه</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>فيسبوك</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/1BDUXPa3VV/</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>رابط صفحة فيسبوك</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>إعلان</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>شريط إعلان أعلى الصفحة (اتركه فارغاً لإخفائه)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>التوصيل</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>نعم</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>نعم أو لا</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>

</xml_diff>